<commit_message>
test to see if ignore works
</commit_message>
<xml_diff>
--- a/trainingen_scored.xlsx
+++ b/trainingen_scored.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH6"/>
+  <dimension ref="A1:AH3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -610,41 +610,123 @@
         </is>
       </c>
       <c r="C2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>AuthenticationError: Error code: 401 - {'type': 'error', 'error': {'type': 'authentication_error', 'message': 'invalid x-api-key'}, 'request_id': 'req_011Ccy4QBBqaXhcz7UecwXFy'}</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PHP Professional leert (junior) developers programmeren in PHP, van functioneel naar object-georiënteerd, met MySQL-database-implementatie, en levert een zelf gebouwde webapplicatie (praktijkcase webwinkel) op.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>expliciet</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>75</v>
+      </c>
+      <c r="J2" t="n">
+        <v>60</v>
+      </c>
+      <c r="K2" t="n">
+        <v>72</v>
+      </c>
+      <c r="L2" t="n">
+        <v>58</v>
+      </c>
+      <c r="M2" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>additief</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>-6</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>PHP zelf is niet verouderd, maar de bron mist elke verwijzing naar de moderne PHP-ecosystem-standaarden (Composer, PSR-autoloading/PSR-standaarden, namespaces, moderne PHP 8.x-taalfeatures zoals typed properties, enums, match, attributes) die in een actuele 'PHP Professional'-opleiding verwacht worden.</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Geen vermelding van Composer/package management | Geen vermelding van PSR-standaarden of namespaces | Geen vermelding van moderne PHP 8.x taalfeatures (enums, match, attributes, typed properties) | phpMyAdmin en klassieke MySQL-scripting worden genoemd zonder moderne database-abstractie (PDO/ORM) context</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>refresh: voeg moderne PHP-ecosysteemonderdelen toe (Composer, PSR-4 autoloading, namespaces, PHP 8.x taalfeatures) aan de OO-module en check of MySQL-module PDO/prepared statements benoemt in plaats van alleen klassieke queries.</t>
+        </is>
+      </c>
+      <c r="T2" t="n">
+        <v>58</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>redelijk</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>afleidbaar</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>aanwezig</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>aanwezig</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>afleidbaar</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>afleidbaar</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>aanwezig</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>Resultaat-sectie met expliciete leeruitkomst (zelfstandig webapplicatie bouwen) | Praktijkcase webwinkel als rode draad | Vier modules met concrete sub-onderwerpen: Inleiding programmeren (array's, regex, cookies, sessies, exception handling, debugging), MySQL, OO programmeren (classes/objects, exception handling, design patterns) | Security als doorlopend thema (input-validatie, veilige database-toegang) | Eindopdracht/praktijkproject als afsluiting | Lijst competenties/vaardigheden (PHP scripts ontwerpen, OOP-basis, relationele databases, phpMyAdmin)</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>Marketing-intro over PHP als 'belangrijke programmeertaal' en WordPress/Magento-voorbeelden (tool-achtergrond, geen leerinhoud) | Sectie 'Cursus PHP: Alternatief' over andere cursussen (Cursus PHP voor programmeurs, Masterclass PHP) — hoort niet bij dit programma | Specialisaties-lijst (Laravel, Symfony, CodeIgniter, WordPress, Drupal) — lijkt eerder verwijzing naar vervolgtrainingen dan onderdeel van dit 5-daagse programma | Disclaimer-zin over 'kan afwijken, bel ons voor actuele inhoud'</t>
+        </is>
+      </c>
       <c r="AD2" t="inlineStr"/>
       <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
+      <c r="AF2" t="b">
+        <v>0</v>
+      </c>
       <c r="AG2" t="inlineStr"/>
       <c r="AH2" t="inlineStr"/>
     </row>
@@ -658,187 +740,121 @@
         </is>
       </c>
       <c r="C3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>AuthenticationError: Error code: 401 - {'type': 'error', 'error': {'type': 'authentication_error', 'message': 'invalid x-api-key'}, 'request_id': 'req_011Ccy4QCFazbdmRz9n4md7u'}</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>6-daagse hands-on cursus waarin developers een VB.NET-applicatie (web én desktop) leren bouwen met Visual Studio en een SQL Server-database, inclusief OOP-principes en databaseontwerp.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>expliciet</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>70</v>
+      </c>
+      <c r="J3" t="n">
+        <v>65</v>
+      </c>
+      <c r="K3" t="n">
+        <v>55</v>
+      </c>
+      <c r="L3" t="n">
+        <v>35</v>
+      </c>
+      <c r="M3" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>structureel</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>-8</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>VB.NET is sinds 2020 door Microsoft 'feature-complete' verklaard (geen taalevolutie meer) en de markt/vraag naar VB.NET is sterk gekrompen; C# is het geadviseerde alternatief voor nieuwe ontwikkeling. Belangrijker: de kernmodule voor webontwikkeling (Web Forms/Server Controls) is een technologie die Microsoft expliciet heeft uitgesloten van ASP.NET Core en 'geen optie meer voor nieuwe ontwikkeling' noemt; alle nieuwe .NET-webontwikkeling gaat naar ASP.NET Core/MVC/Blazor, dat geen Web Forms kent.</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>VB.NET is sinds .NET 5 (2020) in 'maintenance mode': Microsoft evolueert de taal niet meer verder | ASP.NET Web Forms (kernonderdeel van de webmodule) draait alleen op klassiek .NET Framework en is niet beschikbaar/ondersteund in .NET Core/.NET 5+; het wordt gekenschetst als 'shunned but not dead' en 'no longer an option for new development' | Industrieadvies is structureel om voor nieuwe ontwikkeling C# (en ASP.NET Core/Blazor) te gebruiken in plaats van VB.NET/Web Forms | De cursus positioneert VB.NET+Web Forms nog als 'Professional'-traject voor het bouwen van nieuwe applicaties, terwijl dit in de huidige praktijk vrijwel uitsluitend legacy-onderhoud betreft</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>BESLISSING NODIG: bepaal of deze training wordt herpositioneerd (a) als moderne .NET-ontwikkeling (C#/ASP.NET Core/Blazor) met VB.NET als optie, of (b) expliciet als legacy/onderhoudstraining voor bestaande VB.NET/Web Forms-systemen. Dit raakt de kern van het programma (met name de Web Forms-module) en kan niet automatisch uit de bron worden afgeleid.</t>
+        </is>
+      </c>
+      <c r="T3" t="n">
+        <v>40</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>dun</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>afleidbaar</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>aanwezig</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>aanwezig</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>afwezig</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>afwezig</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>afleidbaar</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>Modulebeschrijving 'Programmeren VB.NET': variabelen, loops, functies, commando's, OOP-basis (klassen/objecten), ASP.NET-applicatie-opbouw | Modulebeschrijving 'Visual Studio': werken in de IDE, applicatie volledig opzetten en uitwerken | Modulebeschrijving 'Web Forms en Server Controls': Web Forms als bouwsteen, HTML-/webcontrols, validatie, events, eigen controls maken | Modulebeschrijving 'Windows applicaties voor de desktop': Windows Forms, menu/toolbar/statusbar, setup bouwen | Modulebeschrijving 'Relationele databases': theorie, zelf een databasemodel ontwerpen en implementeren in SQL Server, SQL-query's schrijven, koppeling met VB.NET | Eindcasus-module: zelfgekozen project (web of desktop) met begeleiding — goed bruikbaar als praktijkopdracht/toetsmoment in nieuwe stijl</t>
+        </is>
+      </c>
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="inlineStr"/>
       <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
+      <c r="AF3" t="b">
+        <v>1</v>
+      </c>
       <c r="AG3" t="inlineStr"/>
       <c r="AH3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Opleiding Java Professional</t>
-        </is>
-      </c>
-      <c r="C4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>AuthenticationError: Error code: 401 - {'type': 'error', 'error': {'type': 'authentication_error', 'message': 'invalid x-api-key'}, 'request_id': 'req_011Ccy4QDMoycPAzmEmvuWYQ'}</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>10</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Masterclass PHP</t>
-        </is>
-      </c>
-      <c r="C5" t="b">
-        <v>0</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>AuthenticationError: Error code: 401 - {'type': 'error', 'error': {'type': 'authentication_error', 'message': 'invalid x-api-key'}, 'request_id': 'req_011Ccy4QESJUUcE7tBZNqzRU'}</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>12</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Training Linux</t>
-        </is>
-      </c>
-      <c r="C6" t="b">
-        <v>0</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>AuthenticationError: Error code: 401 - {'type': 'error', 'error': {'type': 'authentication_error', 'message': 'invalid x-api-key'}, 'request_id': 'req_011Ccy4QFVoJeNXEESrHAj4y'}</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr"/>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
nieuwe rubric en error handling voor token limieten
</commit_message>
<xml_diff>
--- a/trainingen_scored.xlsx
+++ b/trainingen_scored.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH3"/>
+  <dimension ref="A1:AB2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -536,65 +536,35 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>dekking_korte_omschrijving</t>
+          <t>bruikbaar</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>dekking_algemene_omschrijving</t>
+          <t>strippen</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>dekking_programma</t>
+          <t>gaten</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>dekking_doelgroep</t>
+          <t>rewrite_guidance</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>dekking_voorkennis</t>
+          <t>menselijke_input_nodig</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>dekking_doelen</t>
+          <t>menselijke_input_wat</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>bruikbaar</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>strippen</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>gaten</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>rewrite_guidance</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>menselijke_input_nodig</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>menselijke_input_wat</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>scorer_confidence</t>
         </is>
@@ -602,11 +572,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Opleiding PHP Professional</t>
+          <t>Opleiding Java Professional</t>
         </is>
       </c>
       <c r="C2" t="b">
@@ -615,7 +585,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PHP Professional leert (junior) developers programmeren in PHP, van functioneel naar object-georiënteerd, met MySQL-database-implementatie, en levert een zelf gebouwde webapplicatie (praktijkcase webwinkel) op.</t>
+          <t>Uitgebreide 11-daagse opleiding tot professioneel Java-programmeur: van taalfundamenten tot objectgeoriënteerd ontwerpen, geavanceerde collections/lambda's, concurrency en JDBC, met een praktijkexamencase en optionele aansluiting op het Oracle Java SE 8 certificaat.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -624,7 +594,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -632,19 +602,19 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="J2" t="n">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="K2" t="n">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="L2" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="M2" t="n">
-        <v>64.2</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -661,21 +631,21 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>PHP zelf is niet verouderd, maar de bron mist elke verwijzing naar de moderne PHP-ecosystem-standaarden (Composer, PSR-autoloading/PSR-standaarden, namespaces, moderne PHP 8.x-taalfeatures zoals typed properties, enums, match, attributes) die in een actuele 'PHP Professional'-opleiding verwacht worden.</t>
+          <t>De opleiding richt zich op Oracle Certified Professional Java SE 8 Programmer, een certificaat dat Oracle inmiddels heeft vervangen door certificeringen op basis van recentere Java-versies (o.a. Java SE 11/17/21). Ook ontbreken taalvernieuwingen sinds Java 9 (var, modules, records, sealed classes, pattern matching, switch-expressions, virtual threads/Project Loom) die inmiddels standaard in Java-opleidingen worden behandeld.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Geen vermelding van Composer/package management | Geen vermelding van PSR-standaarden of namespaces | Geen vermelding van moderne PHP 8.x taalfeatures (enums, match, attributes, typed properties) | phpMyAdmin en klassieke MySQL-scripting worden genoemd zonder moderne database-abstractie (PDO/ORM) context</t>
+          <t>Java SE 8 certificaat is door Oracle uitgefaseerd/vervangen door nieuwere versies | Geen vermelding van taalfeatures uit Java 9-21 (var, records, sealed classes, pattern matching, modules, virtual threads) | Concurrency-module vermeldt geen moderne structured concurrency/virtual threads (Project Loom)</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>refresh: voeg moderne PHP-ecosysteemonderdelen toe (Composer, PSR-4 autoloading, namespaces, PHP 8.x taalfeatures) aan de OO-module en check of MySQL-module PDO/prepared statements benoemt in plaats van alleen klassieke queries.</t>
+          <t>refresh: actualiseer de certificaatverwijzing naar de huidige Oracle Java-certificering, en breid het programma uit met relevante taalvernieuwingen (var, records, sealed classes, pattern matching, modules) en moderne concurrency-concepten, zonder de kernstructuur (fundamenten -&gt; OOP -&gt; verdieping) te wijzigen.</t>
         </is>
       </c>
       <c r="T2" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
@@ -684,177 +654,33 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>afleidbaar</t>
+          <t>Gedetailleerde, gefaseerde modulelijst van fundamenten naar verdieping (variabelen, operatoren, controlestructuren, OOP basis/verdieping, generics, lambda's, concurrency, I/O, JDBC) | Resultaat-sectie met heldere leeruitkomst ('zelf Java-projecten opzetten en uitvoeren') | Examencase/praktijkopdracht-concept als afsluitend onderdeel | Verwijzing naar Oracle-certificering als extra waardepropositie (na actualisatie)</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>aanwezig</t>
+          <t>Verwijzingen naar 'Oracle Certified Professional Java SE 8 Programmer' zonder actualisatie | Cross-sell 'Alternatief'-sectie (C++/C#) en 'Gerelateerd' linklijst | Generieke marketing-intro over wat Java is</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>aanwezig</t>
+          <t>Expliciete doelgroepbeschrijving (niveau, functie, ervaring) | Expliciete voorkennis-eisen | Moderne Java-taalfeatures (9-21) en actuele certificeringspaden | Concrete leerdoelen per modulecluster in plaats van kale onderwerpsopsomming</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>afleidbaar</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>afleidbaar</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>aanwezig</t>
-        </is>
-      </c>
+          <t>Cluster de lange topic-opsomming in 5-7 herkenbare modules (bv. Java-fundamenten, OOP, Collections &amp; Lambda, Concurrency &amp; I/O, Databases/JDBC, Examenproject) passend bij 11 dagen. Formuleer per cluster leeruitkomsten in plaats van kale topic-lijstjes. Actualiseer de Oracle-certificeringsverwijzing en voeg moderne taalfeatures toe. Leid doelgroep/voorkennis af uit het technische, ontwikkelgerichte karakter (persona A, ervaring met programmeren gewenst maar geen Java-voorkennis vereist).</t>
+        </is>
+      </c>
+      <c r="Z2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>Resultaat-sectie met expliciete leeruitkomst (zelfstandig webapplicatie bouwen) | Praktijkcase webwinkel als rode draad | Vier modules met concrete sub-onderwerpen: Inleiding programmeren (array's, regex, cookies, sessies, exception handling, debugging), MySQL, OO programmeren (classes/objects, exception handling, design patterns) | Security als doorlopend thema (input-validatie, veilige database-toegang) | Eindopdracht/praktijkproject als afsluiting | Lijst competenties/vaardigheden (PHP scripts ontwerpen, OOP-basis, relationele databases, phpMyAdmin)</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>Marketing-intro over PHP als 'belangrijke programmeertaal' en WordPress/Magento-voorbeelden (tool-achtergrond, geen leerinhoud) | Sectie 'Cursus PHP: Alternatief' over andere cursussen (Cursus PHP voor programmeurs, Masterclass PHP) — hoort niet bij dit programma | Specialisaties-lijst (Laravel, Symfony, CodeIgniter, WordPress, Drupal) — lijkt eerder verwijzing naar vervolgtrainingen dan onderdeel van dit 5-daagse programma | Disclaimer-zin over 'kan afwijken, bel ons voor actuele inhoud'</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>7</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Opleiding VB.NET Professional</t>
-        </is>
-      </c>
-      <c r="C3" t="b">
-        <v>1</v>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>6-daagse hands-on cursus waarin developers een VB.NET-applicatie (web én desktop) leren bouwen met Visual Studio en een SQL Server-database, inclusief OOP-principes en databaseontwerp.</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>6</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>expliciet</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
-        <v>70</v>
-      </c>
-      <c r="J3" t="n">
-        <v>65</v>
-      </c>
-      <c r="K3" t="n">
-        <v>55</v>
-      </c>
-      <c r="L3" t="n">
-        <v>35</v>
-      </c>
-      <c r="M3" t="n">
-        <v>57.8</v>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>structureel</t>
-        </is>
-      </c>
-      <c r="P3" t="n">
-        <v>-8</v>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>VB.NET is sinds 2020 door Microsoft 'feature-complete' verklaard (geen taalevolutie meer) en de markt/vraag naar VB.NET is sterk gekrompen; C# is het geadviseerde alternatief voor nieuwe ontwikkeling. Belangrijker: de kernmodule voor webontwikkeling (Web Forms/Server Controls) is een technologie die Microsoft expliciet heeft uitgesloten van ASP.NET Core en 'geen optie meer voor nieuwe ontwikkeling' noemt; alle nieuwe .NET-webontwikkeling gaat naar ASP.NET Core/MVC/Blazor, dat geen Web Forms kent.</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>VB.NET is sinds .NET 5 (2020) in 'maintenance mode': Microsoft evolueert de taal niet meer verder | ASP.NET Web Forms (kernonderdeel van de webmodule) draait alleen op klassiek .NET Framework en is niet beschikbaar/ondersteund in .NET Core/.NET 5+; het wordt gekenschetst als 'shunned but not dead' en 'no longer an option for new development' | Industrieadvies is structureel om voor nieuwe ontwikkeling C# (en ASP.NET Core/Blazor) te gebruiken in plaats van VB.NET/Web Forms | De cursus positioneert VB.NET+Web Forms nog als 'Professional'-traject voor het bouwen van nieuwe applicaties, terwijl dit in de huidige praktijk vrijwel uitsluitend legacy-onderhoud betreft</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>BESLISSING NODIG: bepaal of deze training wordt herpositioneerd (a) als moderne .NET-ontwikkeling (C#/ASP.NET Core/Blazor) met VB.NET als optie, of (b) expliciet als legacy/onderhoudstraining voor bestaande VB.NET/Web Forms-systemen. Dit raakt de kern van het programma (met name de Web Forms-module) en kan niet automatisch uit de bron worden afgeleid.</t>
-        </is>
-      </c>
-      <c r="T3" t="n">
-        <v>40</v>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>dun</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>afleidbaar</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>aanwezig</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>aanwezig</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>afwezig</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>afwezig</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>afleidbaar</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>Modulebeschrijving 'Programmeren VB.NET': variabelen, loops, functies, commando's, OOP-basis (klassen/objecten), ASP.NET-applicatie-opbouw | Modulebeschrijving 'Visual Studio': werken in de IDE, applicatie volledig opzetten en uitwerken | Modulebeschrijving 'Web Forms en Server Controls': Web Forms als bouwsteen, HTML-/webcontrols, validatie, events, eigen controls maken | Modulebeschrijving 'Windows applicaties voor de desktop': Windows Forms, menu/toolbar/statusbar, setup bouwen | Modulebeschrijving 'Relationele databases': theorie, zelf een databasemodel ontwerpen en implementeren in SQL Server, SQL-query's schrijven, koppeling met VB.NET | Eindcasus-module: zelfgekozen project (web of desktop) met begeleiding — goed bruikbaar als praktijkopdracht/toetsmoment in nieuwe stijl</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
+          <t>medium</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>